<commit_message>
refactor(oms): 优化 SKU 映射导入逻辑
-移除 SkuMappingWarehouseImportExcelDTO 中的 platformStatusName 字段
- 更新 SkuMappingRuleServiceImpl 中的匹配逻辑
- 移除 SkuMappingWarehouseExcelListener 中关于平台状态的处理
</commit_message>
<xml_diff>
--- a/erp-server/erp-server-oms/src/main/resources/excel/skuMappingWarehouseTemplate.xlsx
+++ b/erp-server/erp-server-oms/src/main/resources/excel/skuMappingWarehouseTemplate.xlsx
@@ -29,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9" uniqueCount="9">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8" uniqueCount="8">
   <si>
     <r>
       <rPr>
@@ -125,9 +125,6 @@
   </si>
   <si>
     <t>账号</t>
-  </si>
-  <si>
-    <t>平台状态</t>
   </si>
 </sst>
 </file>
@@ -1126,8 +1123,8 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:I2"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="13.5" outlineLevelRow="1"/>
+  <dimension ref="A1:H2"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="13.5" outlineLevelRow="1" outlineLevelCol="7"/>
   <cols>
     <col min="1" max="1" width="27.875" style="1" customWidth="1"/>
     <col min="2" max="2" width="20.5083333333333" style="1" customWidth="1"/>
@@ -1139,7 +1136,7 @@
     <col min="8" max="8" width="16.5" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="35.25" customHeight="1" spans="1:9">
+    <row r="1" ht="35.25" customHeight="1" spans="1:8">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -1164,9 +1161,6 @@
       <c r="H1" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="I1" t="s">
-        <v>8</v>
-      </c>
     </row>
     <row r="2" ht="21" customHeight="1" spans="1:6">
       <c r="A2" s="5"/>
@@ -1177,11 +1171,6 @@
       <c r="F2" s="6"/>
     </row>
   </sheetData>
-  <dataValidations count="1">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="I$1:I$1048576">
-      <formula1>"在售,停售,草稿"</formula1>
-    </dataValidation>
-  </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait"/>
   <headerFooter/>

</xml_diff>